<commit_message>
wip: unified repo state for rotation-decomposition bug investigation
</commit_message>
<xml_diff>
--- a/RL/job_logs.xlsx
+++ b/RL/job_logs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -616,6 +616,234 @@
       <c r="O3" t="inlineStr">
         <is>
           <t>2 level hierarchical PPO max steps 75 and 8 envs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-07 22:05:48</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E4" t="n">
+        <v>256</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>92</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>model_jobid_none_film_a</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_none_film_a</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: none | budget_encoding=film | num_envs=2 | budgets=None | n_cycle=1 | n_budget=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-07 22:13:10</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E5" t="n">
+        <v>256</v>
+      </c>
+      <c r="F5" t="n">
+        <v>15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J5" t="n">
+        <v>49</v>
+      </c>
+      <c r="K5" t="n">
+        <v>92</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>model_jobid_none_film_a</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_none_film_a</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: none | budget_encoding=film | num_envs=2 | budgets=None | n_cycle=1 | n_budget=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-08 00:17:22</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E6" t="n">
+        <v>256</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J6" t="n">
+        <v>49</v>
+      </c>
+      <c r="K6" t="n">
+        <v>92</v>
+      </c>
+      <c r="L6" t="n">
+        <v>200000</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>model_jobid_none_film_a</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_none_film_a</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: none | budget_encoding=film | num_envs=8 | budgets=None | n_cycle=1 | n_budget=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-08 04:15:49</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E7" t="n">
+        <v>256</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J7" t="n">
+        <v>49</v>
+      </c>
+      <c r="K7" t="n">
+        <v>92</v>
+      </c>
+      <c r="L7" t="n">
+        <v>200000</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>model_jobid_none_film_b</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_none_film_b</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: none | budget_encoding=film | num_envs=8 | budgets=None | n_cycle=1 | n_budget=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed: 1 rot is happening now
</commit_message>
<xml_diff>
--- a/RL/job_logs.xlsx
+++ b/RL/job_logs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1018,6 +1018,177 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-09 02:14:26</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J11" t="n">
+        <v>33</v>
+      </c>
+      <c r="K11" t="n">
+        <v>92</v>
+      </c>
+      <c r="L11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>model_jobid_lagrangian_od_ov_film_a</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_lagrangian_od_ov_film_a</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: lagrangian_od_ov | budget_encoding=film | num_envs=4 | budgets=None | n_cycle=1 | n_budget=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-09 02:48:08</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E12" t="n">
+        <v>256</v>
+      </c>
+      <c r="F12" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J12" t="n">
+        <v>22526</v>
+      </c>
+      <c r="K12" t="n">
+        <v>92</v>
+      </c>
+      <c r="L12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>model_jobid_lagrangian_od_ov_film_a</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_lagrangian_od_ov_film_a</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: lagrangian_od_ov | budget_encoding=film | num_envs=4 | budgets=None | n_cycle=1 | n_budget=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-09 02:53:01</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E13" t="n">
+        <v>256</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J13" t="n">
+        <v>22526</v>
+      </c>
+      <c r="K13" t="n">
+        <v>92</v>
+      </c>
+      <c r="L13" t="n">
+        <v>200000</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>model_jobid_lagrangian_od_ov_film_b</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_lagrangian_od_ov_film_b</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: lagrangian_od_ov | budget_encoding=film | num_envs=4 | budgets=None | n_cycle=1 | n_budget=5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>